<commit_message>
chore: refresh consort, swimlane, and tabtools demos
Regenerate consort and swimlane PNG demos; demo_swimlane.do installs
tc_schemes and applies scheme(modern) to selected plots.
Add table1_tc and desctab binary small-cell suppression cases to
demo_tabtools.do, regenerating demo workbooks and trimming the Markdown report.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_desctab.xlsx
+++ b/tabtools/demo/demo_desctab.xlsx
@@ -14,13 +14,14 @@
     <sheet name="Custom" sheetId="6" r:id="rId8"/>
     <sheet name="Small Cells Primary" sheetId="7" r:id="rId9"/>
     <sheet name="Small Cells Complement" sheetId="8" r:id="rId10"/>
+    <sheet name="Small Cells Binary" sheetId="9" r:id="rId11"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="288" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="329" uniqueCount="103">
   <si>
     <t>Foreign cars by repair record</t>
   </si>
@@ -309,12 +310,33 @@
   <si>
     <t>20</t>
   </si>
+  <si>
+    <t>Small-cell suppression: binary variable</t>
+  </si>
+  <si>
+    <t>Rare adverse event</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="1258">
+  <fonts count="1451">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -3937,6 +3959,832 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <b/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -5689,7 +6537,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="904">
+  <borders count="1039">
     <border>
       <left/>
       <right/>
@@ -11742,11 +12590,920 @@
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="thin"/>
+      <top style="none"/>
+      <bottom style="thin"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="904">
+  <cellXfs count="1039">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -15219,6 +16976,528 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="0" fontId="1257" fillId="0" borderId="903" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="904" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="905" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="906" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="907" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="908" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="909" xfId="0"/>
+    <xf numFmtId="0" fontId="1259" fillId="0" borderId="910" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1261" fillId="0" borderId="911" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1263" fillId="0" borderId="912" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1265" fillId="0" borderId="913" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1267" fillId="0" borderId="914" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1269" fillId="0" borderId="915" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1271" fillId="0" borderId="916" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1273" fillId="0" borderId="917" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1275" fillId="0" borderId="918" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1277" fillId="0" borderId="919" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1279" fillId="0" borderId="920" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1281" fillId="0" borderId="921" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1283" fillId="0" borderId="922" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1285" fillId="0" borderId="923" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1287" fillId="0" borderId="924" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1289" fillId="0" borderId="925" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1291" fillId="0" borderId="926" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1293" fillId="0" borderId="927" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1295" fillId="0" borderId="928" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1297" fillId="0" borderId="929" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1299" fillId="0" borderId="930" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1301" fillId="0" borderId="931" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1303" fillId="0" borderId="932" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1305" fillId="0" borderId="933" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1307" fillId="0" borderId="934" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1309" fillId="0" borderId="935" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1311" fillId="0" borderId="936" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1313" fillId="0" borderId="937" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1315" fillId="0" borderId="938" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1317" fillId="0" borderId="939" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1319" fillId="0" borderId="940" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1321" fillId="0" borderId="941" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1323" fillId="0" borderId="942" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1325" fillId="0" borderId="943" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1327" fillId="0" borderId="944" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1329" fillId="0" borderId="945" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1331" fillId="0" borderId="946" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1333" fillId="0" borderId="947" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1335" fillId="0" borderId="948" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1337" fillId="0" borderId="949" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1339" fillId="0" borderId="950" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1341" fillId="0" borderId="951" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1343" fillId="0" borderId="952" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1345" fillId="0" borderId="953" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1347" fillId="0" borderId="954" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1348" fillId="0" borderId="955" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1349" fillId="0" borderId="956" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1350" fillId="0" borderId="957" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1352" fillId="0" borderId="958" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1354" fillId="0" borderId="959" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1356" fillId="0" borderId="960" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1358" fillId="0" borderId="961" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1360" fillId="0" borderId="962" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1362" fillId="0" borderId="963" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1364" fillId="0" borderId="964" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1366" fillId="0" borderId="965" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1368" fillId="0" borderId="966" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1370" fillId="0" borderId="967" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1372" fillId="0" borderId="968" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1374" fillId="0" borderId="969" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1376" fillId="0" borderId="970" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1378" fillId="0" borderId="971" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1380" fillId="0" borderId="972" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1382" fillId="0" borderId="973" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1384" fillId="0" borderId="974" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1385" fillId="0" borderId="975" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1386" fillId="0" borderId="976" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1387" fillId="0" borderId="977" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1388" fillId="0" borderId="978" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1389" fillId="0" borderId="979" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1390" fillId="0" borderId="980" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1391" fillId="0" borderId="981" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1392" fillId="0" borderId="982" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1393" fillId="0" borderId="983" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1394" fillId="0" borderId="984" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1395" fillId="0" borderId="985" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1396" fillId="0" borderId="986" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1397" fillId="0" borderId="987" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1398" fillId="0" borderId="988" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1399" fillId="0" borderId="989" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1400" fillId="0" borderId="990" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1401" fillId="0" borderId="991" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1402" fillId="0" borderId="992" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1403" fillId="0" borderId="993" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1404" fillId="0" borderId="994" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1405" fillId="0" borderId="995" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1406" fillId="0" borderId="996" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1407" fillId="0" borderId="997" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1408" fillId="0" borderId="998" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1409" fillId="0" borderId="999" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1410" fillId="0" borderId="1000" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1411" fillId="0" borderId="1001" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1412" fillId="0" borderId="1002" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1413" fillId="0" borderId="1003" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1414" fillId="0" borderId="1004" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1415" fillId="0" borderId="1005" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1416" fillId="0" borderId="1006" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1417" fillId="0" borderId="1007" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1418" fillId="0" borderId="1008" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1419" fillId="0" borderId="1009" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1420" fillId="0" borderId="1010" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1421" fillId="0" borderId="1011" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1422" fillId="0" borderId="1012" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1423" fillId="0" borderId="1013" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1424" fillId="0" borderId="1014" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1425" fillId="0" borderId="1015" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1426" fillId="0" borderId="1016" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1427" fillId="0" borderId="1017" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1428" fillId="0" borderId="1018" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1429" fillId="0" borderId="1019" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1430" fillId="0" borderId="1020" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1431" fillId="0" borderId="1021" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1432" fillId="0" borderId="1022" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1433" fillId="0" borderId="1023" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1434" fillId="0" borderId="1024" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1435" fillId="0" borderId="1025" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1436" fillId="0" borderId="1026" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1437" fillId="0" borderId="1027" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1438" fillId="0" borderId="1028" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1439" fillId="0" borderId="1029" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1440" fillId="0" borderId="1030" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1441" fillId="0" borderId="1031" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1442" fillId="0" borderId="1032" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1443" fillId="0" borderId="1033" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1444" fillId="0" borderId="1034" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1445" fillId="0" borderId="1035" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1446" fillId="0" borderId="1036" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1448" fillId="0" borderId="1037" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1450" fillId="0" borderId="1038" xfId="0" applyNumberFormat="true" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -16373,4 +18652,168 @@
     <mergeCell ref="B9:E9"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="1.7109375" style="904" customWidth="true"/>
+    <col min="2" max="2" width="13.7109375" style="905" customWidth="true"/>
+    <col min="3" max="3" width="20.7109375" style="906" customWidth="true"/>
+    <col min="4" max="4" width="20.7109375" style="907" customWidth="true"/>
+    <col min="5" max="5" width="20.7109375" style="908" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="909" customFormat="true" ht="30" customHeight="true">
+      <c r="A1" s="958" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="950" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="950" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="950" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="950" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="915" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1013" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="988" t="s">
+        <v>97</v>
+      </c>
+      <c r="D2" s="1020" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="1006" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="920" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1014" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="978" t="s">
+        <v>98</v>
+      </c>
+      <c r="D3" s="1021" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="1007" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="925" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1015" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="981" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="1022" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="1008" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="930" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="1016" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="992" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1023" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1009" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="935" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="1017" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="1027" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="1028" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" s="1029" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="940" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="1018" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="1030" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="1031" t="s">
+        <v>88</v>
+      </c>
+      <c r="E7" s="1032" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="945" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="1019" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="1033" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="1034" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="1035" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="1038" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" s="0"/>
+      <c r="D9" s="0"/>
+      <c r="E9" s="0"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B9:E9"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(tabtools): size Excel columns from rendered content
Prevent sparse Excel tables from inheriting the widest sibling column.
Add _tabtools_colwidth.ado for Unicode display-width measurement, per-column
bounds, and wrapped-header sizing; use it in desctab, table1_tc, regtab,
effecttab, and comptab rendering paths.
Bump tabtools to 2.1.3 and sync .ado, .pkg, .sthlp, and README metadata.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_desctab.xlsx
+++ b/tabtools/demo/demo_desctab.xlsx
@@ -961,8 +961,8 @@
   <cols>
     <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
     <col min="2" max="2" width="15.7109375" style="1" customWidth="true"/>
-    <col min="3" max="3" width="14.7109375" style="1" customWidth="true"/>
-    <col min="4" max="4" width="14.7109375" style="1" customWidth="true"/>
+    <col min="3" max="3" width="13.7109375" style="1" customWidth="true"/>
+    <col min="4" max="4" width="13.7109375" style="1" customWidth="true"/>
     <col min="5" max="5" width="10.7109375" style="1" customWidth="true"/>
   </cols>
   <sheetData>
@@ -1156,8 +1156,8 @@
   <cols>
     <col min="1" max="1" width="1.7109375" style="1" customWidth="true"/>
     <col min="2" max="2" width="18.7109375" style="1" customWidth="true"/>
-    <col min="3" max="3" width="13.7109375" style="1" customWidth="true"/>
-    <col min="4" max="4" width="13.7109375" style="1" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" style="1" customWidth="true"/>
+    <col min="4" max="4" width="12.7109375" style="1" customWidth="true"/>
     <col min="5" max="5" width="10.7109375" style="1" customWidth="true"/>
   </cols>
   <sheetData>

</xml_diff>